<commit_message>
Rename vehicle-ownership inputs and refit the car ownership curve
Renames VOS/VOIR to VpHCS/VpHCIR (new trans/VpHC folder) and gives BFfHO and MBFGR
their own folders. Refits the passenger-car curve to the inputs changed in 44c1144e
(saturation 2.17 -> 2.27 vehicles per household).
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\AppData\Local\Temp\claude\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\EPS Structure Research\eps-us-input-rename2\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF0AF5B-A907-47AC-87E4-A9C0CFB9566C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09319B7B-B9B4-4734-B6A5-3E30C1B6365C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1849" uniqueCount="1059">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -3168,19 +3168,37 @@
     <t>Your country has data on vehicle occupancy or load factors, or on how car ownership responds to transit and demand-management policies</t>
   </si>
   <si>
-    <t>VOS</t>
-  </si>
-  <si>
-    <t>Vehicle Ownership Saturation</t>
-  </si>
-  <si>
-    <t>BFfHO BAU Fleet from Household Ownership, VOS Vehicle Ownership Saturation, VOIR Vehicle Ownership Income Response, MBFGR Minimum BAU Fleet Growth Rate</t>
-  </si>
-  <si>
     <t>SYVbT, NoH, BGDP</t>
   </si>
   <si>
-    <t>Your country has a vehicle-stock projection to fit the car-ownership curve to (otherwise use the published Dargay-Gately defaults in the workbook), or vehicle types whose fleet should keep growing on a trend while loading recovers to normal</t>
+    <t>VpHC</t>
+  </si>
+  <si>
+    <t>Vehicles per Household Curve</t>
+  </si>
+  <si>
+    <t>VpHCS Vehicles per Household Curve Saturation, VpHCIR Vehicles per Household Curve Income Response</t>
+  </si>
+  <si>
+    <t>Your country has a vehicle-stock projection to fit the car-ownership curve to; otherwise use the published Dargay-Gately values in the workbook, converted to per household and to your GDP units</t>
+  </si>
+  <si>
+    <t>BFfHO</t>
+  </si>
+  <si>
+    <t>BAU Fleet from Household Ownership</t>
+  </si>
+  <si>
+    <t>A vehicle type other than passenger cars should follow households x ownership rather than travel at normal use</t>
+  </si>
+  <si>
+    <t>MBFGR</t>
+  </si>
+  <si>
+    <t>Minimum BAU Fleet Growth Rate</t>
+  </si>
+  <si>
+    <t>A vehicle type that fills toward its normal loading (buses, passenger rail, aircraft) should keep growing on an observed fleet trend meanwhile</t>
   </si>
 </sst>
 </file>
@@ -3994,7 +4012,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G392"/>
+  <dimension ref="A1:G394"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.5703125" style="2" customWidth="1"/>
@@ -9902,32 +9920,34 @@
         <v>765</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>788</v>
+        <v>1053</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>789</v>
+        <v>1054</v>
       </c>
       <c r="D330" s="7"/>
       <c r="E330" s="7"/>
       <c r="F330" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G330" s="26"/>
-    </row>
-    <row r="331" spans="1:7" ht="30" customHeight="1">
+        <v>29</v>
+      </c>
+      <c r="G330" s="26" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7">
       <c r="A331" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="D331" s="7"/>
       <c r="E331" s="7"/>
       <c r="F331" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G331" s="26"/>
     </row>
@@ -9936,97 +9956,97 @@
         <v>765</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>793</v>
-      </c>
-      <c r="D332" s="1"/>
+        <v>791</v>
+      </c>
+      <c r="D332" s="7"/>
       <c r="E332" s="7"/>
       <c r="F332" s="5" t="s">
         <v>20</v>
       </c>
       <c r="G332" s="26"/>
     </row>
-    <row r="333" spans="1:7" ht="60" customHeight="1">
+    <row r="333" spans="1:7" ht="30" customHeight="1">
       <c r="A333" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>795</v>
-      </c>
-      <c r="D333" s="7"/>
+        <v>793</v>
+      </c>
+      <c r="D333" s="1"/>
       <c r="E333" s="7"/>
       <c r="F333" s="5" t="s">
         <v>20</v>
       </c>
       <c r="G333" s="26"/>
     </row>
-    <row r="334" spans="1:7">
+    <row r="334" spans="1:7" ht="60" customHeight="1">
       <c r="A334" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="D334" s="7"/>
       <c r="E334" s="7"/>
-      <c r="F334" s="3" t="s">
+      <c r="F334" s="5" t="s">
         <v>20</v>
       </c>
       <c r="G334" s="26"/>
     </row>
-    <row r="335" spans="1:7" ht="60" customHeight="1">
+    <row r="335" spans="1:7">
       <c r="A335" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>799</v>
-      </c>
-      <c r="D335" s="7" t="s">
-        <v>800</v>
-      </c>
+        <v>797</v>
+      </c>
+      <c r="D335" s="7"/>
       <c r="E335" s="7"/>
       <c r="F335" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G335" s="26"/>
     </row>
-    <row r="336" spans="1:7" ht="45" customHeight="1">
+    <row r="336" spans="1:7" ht="60" customHeight="1">
       <c r="A336" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>802</v>
-      </c>
-      <c r="D336" s="7"/>
+        <v>799</v>
+      </c>
+      <c r="D336" s="7" t="s">
+        <v>800</v>
+      </c>
       <c r="E336" s="7"/>
       <c r="F336" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G336" s="26"/>
     </row>
-    <row r="337" spans="1:7" ht="60" customHeight="1">
+    <row r="337" spans="1:7" ht="45" customHeight="1">
       <c r="A337" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="D337" s="7"/>
       <c r="E337" s="7"/>
@@ -10035,32 +10055,32 @@
       </c>
       <c r="G337" s="26"/>
     </row>
-    <row r="338" spans="1:7">
+    <row r="338" spans="1:7" ht="60" customHeight="1">
       <c r="A338" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="D338" s="7"/>
       <c r="E338" s="7"/>
-      <c r="F338" s="4" t="s">
-        <v>10</v>
+      <c r="F338" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="G338" s="26"/>
     </row>
-    <row r="339" spans="1:7" ht="30" customHeight="1">
+    <row r="339" spans="1:7">
       <c r="A339" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D339" s="7"/>
       <c r="E339" s="7"/>
@@ -10074,61 +10094,61 @@
         <v>765</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D340" s="7"/>
       <c r="E340" s="7"/>
-      <c r="F340" s="6" t="s">
+      <c r="F340" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G340" s="24"/>
-    </row>
-    <row r="341" spans="1:7">
+      <c r="G340" s="26"/>
+    </row>
+    <row r="341" spans="1:7" ht="30" customHeight="1">
       <c r="A341" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="D341" s="7"/>
       <c r="E341" s="7"/>
-      <c r="F341" s="5" t="s">
+      <c r="F341" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G341" s="26"/>
-    </row>
-    <row r="342" spans="1:7" ht="60" customHeight="1">
+      <c r="G341" s="24"/>
+    </row>
+    <row r="342" spans="1:7">
       <c r="A342" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="D342" s="7"/>
       <c r="E342" s="7"/>
       <c r="F342" s="5" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G342" s="26"/>
     </row>
-    <row r="343" spans="1:7">
+    <row r="343" spans="1:7" ht="60" customHeight="1">
       <c r="A343" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="D343" s="7"/>
       <c r="E343" s="7"/>
@@ -10142,50 +10162,50 @@
         <v>765</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D344" s="7"/>
       <c r="E344" s="7"/>
-      <c r="F344" s="4" t="s">
-        <v>819</v>
-      </c>
-      <c r="G344" s="26" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="345" spans="1:7" ht="45" customHeight="1">
+      <c r="F344" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G344" s="26"/>
+    </row>
+    <row r="345" spans="1:7">
       <c r="A345" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>822</v>
-      </c>
-      <c r="D345" s="1"/>
+        <v>818</v>
+      </c>
+      <c r="D345" s="7"/>
       <c r="E345" s="7"/>
-      <c r="F345" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G345" s="26"/>
-    </row>
-    <row r="346" spans="1:7">
+      <c r="F345" s="4" t="s">
+        <v>819</v>
+      </c>
+      <c r="G345" s="26" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" ht="45" customHeight="1">
       <c r="A346" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>824</v>
-      </c>
-      <c r="D346" s="7"/>
+        <v>822</v>
+      </c>
+      <c r="D346" s="1"/>
       <c r="E346" s="7"/>
-      <c r="F346" s="4" t="s">
+      <c r="F346" s="5" t="s">
         <v>20</v>
       </c>
       <c r="G346" s="26"/>
@@ -10195,53 +10215,53 @@
         <v>765</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>1044</v>
+        <v>823</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>1045</v>
-      </c>
-      <c r="D347" s="7" t="s">
-        <v>1046</v>
-      </c>
+        <v>824</v>
+      </c>
+      <c r="D347" s="7"/>
       <c r="E347" s="7"/>
-      <c r="F347" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G347" s="26" t="s">
-        <v>1047</v>
-      </c>
+      <c r="F347" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G347" s="26"/>
     </row>
     <row r="348" spans="1:7">
       <c r="A348" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>825</v>
+        <v>1044</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="D348" s="7"/>
+        <v>1045</v>
+      </c>
+      <c r="D348" s="7" t="s">
+        <v>1046</v>
+      </c>
       <c r="E348" s="7"/>
-      <c r="F348" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G348" s="26"/>
-    </row>
-    <row r="349" spans="1:7" ht="45" customHeight="1">
+      <c r="F348" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G348" s="26" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7">
       <c r="A349" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="D349" s="7"/>
       <c r="E349" s="7"/>
-      <c r="F349" s="5" t="s">
-        <v>29</v>
+      <c r="F349" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="G349" s="26"/>
     </row>
@@ -10250,85 +10270,85 @@
         <v>765</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="D350" s="7" t="s">
-        <v>831</v>
-      </c>
+        <v>828</v>
+      </c>
+      <c r="D350" s="7"/>
       <c r="E350" s="7"/>
-      <c r="F350" s="3" t="s">
-        <v>20</v>
+      <c r="F350" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="G350" s="26"/>
     </row>
-    <row r="351" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
+    <row r="351" spans="1:7" ht="45" customHeight="1">
       <c r="A351" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>833</v>
-      </c>
-      <c r="D351" s="7"/>
+        <v>830</v>
+      </c>
+      <c r="D351" s="7" t="s">
+        <v>831</v>
+      </c>
       <c r="E351" s="7"/>
       <c r="F351" s="3" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G351" s="26"/>
     </row>
-    <row r="352" spans="1:7" ht="45" customHeight="1">
+    <row r="352" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
       <c r="A352" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="D352" s="7"/>
       <c r="E352" s="7"/>
-      <c r="F352" s="5" t="s">
+      <c r="F352" s="3" t="s">
         <v>29</v>
       </c>
       <c r="G352" s="26"/>
     </row>
-    <row r="353" spans="1:7" ht="30">
+    <row r="353" spans="1:7" ht="45" customHeight="1">
       <c r="A353" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="D353" s="7"/>
       <c r="E353" s="7"/>
-      <c r="F353" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G353" s="24"/>
-    </row>
-    <row r="354" spans="1:7" ht="30" customHeight="1">
+      <c r="F353" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G353" s="26"/>
+    </row>
+    <row r="354" spans="1:7" ht="30">
       <c r="A354" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="D354" s="7"/>
       <c r="E354" s="7"/>
       <c r="F354" s="16" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G354" s="24"/>
     </row>
@@ -10337,10 +10357,10 @@
         <v>765</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="D355" s="7"/>
       <c r="E355" s="7"/>
@@ -10349,70 +10369,68 @@
       </c>
       <c r="G355" s="24"/>
     </row>
-    <row r="356" spans="1:7">
+    <row r="356" spans="1:7" ht="30" customHeight="1">
       <c r="A356" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="D356" s="7"/>
-      <c r="E356" s="1"/>
-      <c r="F356" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G356" s="26"/>
+      <c r="E356" s="7"/>
+      <c r="F356" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G356" s="24"/>
     </row>
     <row r="357" spans="1:7">
       <c r="A357" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="D357" s="7"/>
-      <c r="E357" s="7"/>
-      <c r="F357" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G357" s="26" t="s">
-        <v>846</v>
-      </c>
-    </row>
-    <row r="358" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
+      <c r="E357" s="1"/>
+      <c r="F357" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G357" s="26"/>
+    </row>
+    <row r="358" spans="1:7">
       <c r="A358" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="D358" s="7"/>
       <c r="E358" s="7"/>
-      <c r="F358" s="4" t="s">
+      <c r="F358" s="5" t="s">
         <v>14</v>
       </c>
       <c r="G358" s="26" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="359" spans="1:7" ht="45" customHeight="1">
+    <row r="359" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
       <c r="A359" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B359" s="2" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="D359" s="7"/>
       <c r="E359" s="7"/>
@@ -10423,230 +10441,234 @@
         <v>846</v>
       </c>
     </row>
-    <row r="360" spans="1:7" ht="30" customHeight="1">
+    <row r="360" spans="1:7" ht="45" customHeight="1">
       <c r="A360" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B360" s="2" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="D360" s="7"/>
-      <c r="E360" s="7" t="s">
-        <v>796</v>
-      </c>
-      <c r="F360" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G360" s="24"/>
-    </row>
-    <row r="361" spans="1:7" ht="45" customHeight="1">
+      <c r="E360" s="7"/>
+      <c r="F360" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G360" s="26" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="361" spans="1:7">
       <c r="A361" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>853</v>
+        <v>1056</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>854</v>
+        <v>1057</v>
       </c>
       <c r="D361" s="7"/>
       <c r="E361" s="7"/>
       <c r="F361" s="5" t="s">
-        <v>855</v>
-      </c>
-      <c r="G361" s="26"/>
-    </row>
-    <row r="362" spans="1:7" ht="45" customHeight="1">
+        <v>29</v>
+      </c>
+      <c r="G361" s="26" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="362" spans="1:7" ht="30" customHeight="1">
       <c r="A362" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B362" s="2" t="s">
-        <v>1005</v>
+        <v>851</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>1006</v>
+        <v>852</v>
       </c>
       <c r="D362" s="7"/>
-      <c r="E362" s="7"/>
-      <c r="F362" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G362" s="26"/>
-    </row>
-    <row r="363" spans="1:7" ht="30">
+      <c r="E362" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="F362" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G362" s="24"/>
+    </row>
+    <row r="363" spans="1:7" ht="45" customHeight="1">
       <c r="A363" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B363" s="2" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="C363" s="2" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="D363" s="7"/>
       <c r="E363" s="7"/>
       <c r="F363" s="5" t="s">
-        <v>29</v>
+        <v>855</v>
       </c>
       <c r="G363" s="26"/>
     </row>
-    <row r="364" spans="1:7" ht="30" customHeight="1">
+    <row r="364" spans="1:7" ht="45" customHeight="1">
       <c r="A364" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B364" s="2" t="s">
-        <v>858</v>
+        <v>1005</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>859</v>
+        <v>1006</v>
       </c>
       <c r="D364" s="7"/>
       <c r="E364" s="7"/>
-      <c r="F364" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G364" s="24"/>
-    </row>
-    <row r="365" spans="1:7" ht="30" customHeight="1">
+      <c r="F364" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G364" s="26"/>
+    </row>
+    <row r="365" spans="1:7" ht="30">
       <c r="A365" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B365" s="2" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="D365" s="7"/>
       <c r="E365" s="7"/>
-      <c r="F365" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="G365" s="26" t="s">
-        <v>862</v>
-      </c>
-    </row>
-    <row r="366" spans="1:7">
+      <c r="F365" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G365" s="26"/>
+    </row>
+    <row r="366" spans="1:7" ht="30" customHeight="1">
       <c r="A366" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B366" s="2" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="D366" s="7"/>
       <c r="E366" s="7"/>
-      <c r="F366" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G366" s="26"/>
-    </row>
-    <row r="367" spans="1:7">
+      <c r="F366" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G366" s="24"/>
+    </row>
+    <row r="367" spans="1:7" ht="30" customHeight="1">
       <c r="A367" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="D367" s="7"/>
       <c r="E367" s="7"/>
-      <c r="F367" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G367" s="26"/>
-    </row>
-    <row r="368" spans="1:7" ht="30" customHeight="1">
+      <c r="F367" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G367" s="26" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="368" spans="1:7">
       <c r="A368" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>867</v>
+        <v>863</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="D368" s="7"/>
       <c r="E368" s="7"/>
       <c r="F368" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G368" s="26" t="s">
-        <v>869</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G368" s="26"/>
     </row>
     <row r="369" spans="1:7">
       <c r="A369" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="D369" s="7"/>
       <c r="E369" s="7"/>
-      <c r="F369" s="12" t="s">
+      <c r="F369" s="4" t="s">
         <v>20</v>
       </c>
       <c r="G369" s="26"/>
     </row>
-    <row r="370" spans="1:7">
-      <c r="A370" t="s">
+    <row r="370" spans="1:7" ht="30" customHeight="1">
+      <c r="A370" s="2" t="s">
         <v>765</v>
       </c>
-      <c r="B370" t="s">
-        <v>872</v>
-      </c>
-      <c r="C370" t="s">
-        <v>873</v>
+      <c r="B370" s="2" t="s">
+        <v>867</v>
+      </c>
+      <c r="C370" s="2" t="s">
+        <v>868</v>
       </c>
       <c r="D370" s="7"/>
       <c r="E370" s="7"/>
-      <c r="F370" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G370" s="26"/>
+      <c r="F370" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G370" s="26" t="s">
+        <v>869</v>
+      </c>
     </row>
     <row r="371" spans="1:7">
       <c r="A371" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B371" s="2" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>875</v>
+        <v>871</v>
       </c>
       <c r="D371" s="7"/>
-      <c r="E371" s="1"/>
-      <c r="F371" s="5" t="s">
+      <c r="E371" s="7"/>
+      <c r="F371" s="12" t="s">
         <v>20</v>
       </c>
       <c r="G371" s="26"/>
     </row>
     <row r="372" spans="1:7">
-      <c r="A372" s="2" t="s">
+      <c r="A372" t="s">
         <v>765</v>
       </c>
-      <c r="B372" s="2" t="s">
-        <v>876</v>
-      </c>
-      <c r="C372" s="2" t="s">
-        <v>877</v>
+      <c r="B372" t="s">
+        <v>872</v>
+      </c>
+      <c r="C372" t="s">
+        <v>873</v>
       </c>
       <c r="D372" s="7"/>
       <c r="E372" s="7"/>
-      <c r="F372" s="5" t="s">
-        <v>37</v>
+      <c r="F372" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="G372" s="26"/>
     </row>
@@ -10655,15 +10677,13 @@
         <v>765</v>
       </c>
       <c r="B373" s="2" t="s">
-        <v>1007</v>
+        <v>874</v>
       </c>
       <c r="C373" s="2" t="s">
-        <v>1008</v>
+        <v>875</v>
       </c>
       <c r="D373" s="7"/>
-      <c r="E373" s="7" t="s">
-        <v>1009</v>
-      </c>
+      <c r="E373" s="1"/>
       <c r="F373" s="5" t="s">
         <v>20</v>
       </c>
@@ -10674,15 +10694,15 @@
         <v>765</v>
       </c>
       <c r="B374" s="2" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="D374" s="7"/>
       <c r="E374" s="7"/>
-      <c r="F374" s="4" t="s">
-        <v>96</v>
+      <c r="F374" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="G374" s="26"/>
     </row>
@@ -10691,163 +10711,163 @@
         <v>765</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>880</v>
+        <v>1007</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>881</v>
+        <v>1008</v>
       </c>
       <c r="D375" s="7"/>
       <c r="E375" s="7" t="s">
-        <v>876</v>
-      </c>
-      <c r="F375" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="F375" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G375" s="24"/>
+      <c r="G375" s="26"/>
     </row>
     <row r="376" spans="1:7">
       <c r="A376" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="D376" s="7"/>
       <c r="E376" s="7"/>
-      <c r="F376" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G376" s="24"/>
+      <c r="F376" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G376" s="26"/>
     </row>
     <row r="377" spans="1:7">
       <c r="A377" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B377" s="2" t="s">
-        <v>1048</v>
+        <v>880</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>1049</v>
-      </c>
-      <c r="D377" s="7" t="s">
-        <v>1050</v>
-      </c>
+        <v>881</v>
+      </c>
+      <c r="D377" s="7"/>
       <c r="E377" s="7" t="s">
-        <v>1051</v>
-      </c>
-      <c r="F377" s="5" t="s">
+        <v>876</v>
+      </c>
+      <c r="F377" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="G377" s="26" t="s">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="378" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A378" s="17" t="s">
+      <c r="G377" s="24"/>
+    </row>
+    <row r="378" spans="1:7">
+      <c r="A378" s="2" t="s">
         <v>765</v>
       </c>
-      <c r="B378" s="17" t="s">
-        <v>884</v>
-      </c>
-      <c r="C378" s="17" t="s">
-        <v>885</v>
-      </c>
-      <c r="D378" s="27"/>
-      <c r="E378" s="27"/>
-      <c r="F378" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="G378" s="28"/>
+      <c r="B378" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="C378" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="D378" s="7"/>
+      <c r="E378" s="7"/>
+      <c r="F378" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="G378" s="24"/>
     </row>
     <row r="379" spans="1:7">
       <c r="A379" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B379" s="2" t="s">
-        <v>886</v>
+        <v>1049</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>887</v>
-      </c>
-      <c r="D379" s="1"/>
-      <c r="E379" s="7"/>
+        <v>1050</v>
+      </c>
+      <c r="D379" s="7" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E379" s="7" t="s">
+        <v>1048</v>
+      </c>
       <c r="F379" s="5" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G379" s="26" t="s">
-        <v>888</v>
-      </c>
-    </row>
-    <row r="380" spans="1:7">
-      <c r="A380" s="2" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A380" s="17" t="s">
         <v>765</v>
       </c>
-      <c r="B380" s="2" t="s">
-        <v>889</v>
-      </c>
-      <c r="C380" s="2" t="s">
-        <v>890</v>
-      </c>
-      <c r="D380" s="1"/>
-      <c r="E380" s="7"/>
-      <c r="F380" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G380" s="26" t="s">
-        <v>891</v>
-      </c>
-    </row>
-    <row r="381" spans="1:7" ht="30">
+      <c r="B380" s="17" t="s">
+        <v>884</v>
+      </c>
+      <c r="C380" s="17" t="s">
+        <v>885</v>
+      </c>
+      <c r="D380" s="27"/>
+      <c r="E380" s="27"/>
+      <c r="F380" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="G380" s="28"/>
+    </row>
+    <row r="381" spans="1:7">
       <c r="A381" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B381" s="2" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>893</v>
+        <v>887</v>
       </c>
       <c r="D381" s="1"/>
       <c r="E381" s="7"/>
       <c r="F381" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G381" s="26"/>
+        <v>10</v>
+      </c>
+      <c r="G381" s="26" t="s">
+        <v>888</v>
+      </c>
     </row>
     <row r="382" spans="1:7">
       <c r="A382" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B382" s="2" t="s">
-        <v>1010</v>
+        <v>889</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>1011</v>
+        <v>890</v>
       </c>
       <c r="D382" s="1"/>
       <c r="E382" s="7"/>
       <c r="F382" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G382" s="26"/>
-    </row>
-    <row r="383" spans="1:7">
+        <v>14</v>
+      </c>
+      <c r="G382" s="26" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" ht="30">
       <c r="A383" s="2" t="s">
         <v>765</v>
       </c>
       <c r="B383" s="2" t="s">
-        <v>1012</v>
+        <v>892</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>1013</v>
+        <v>893</v>
       </c>
       <c r="D383" s="1"/>
-      <c r="E383" s="7" t="s">
-        <v>772</v>
-      </c>
+      <c r="E383" s="7"/>
       <c r="F383" s="5" t="s">
         <v>29</v>
       </c>
@@ -10858,10 +10878,10 @@
         <v>765</v>
       </c>
       <c r="B384" s="2" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="D384" s="1"/>
       <c r="E384" s="7"/>
@@ -10872,137 +10892,173 @@
     </row>
     <row r="385" spans="1:7">
       <c r="A385" s="2" t="s">
-        <v>894</v>
+        <v>765</v>
       </c>
       <c r="B385" s="2" t="s">
-        <v>895</v>
+        <v>1012</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>896</v>
-      </c>
-      <c r="D385" s="7" t="s">
-        <v>897</v>
-      </c>
-      <c r="E385" s="7"/>
-      <c r="F385" s="25" t="s">
-        <v>20</v>
+        <v>1013</v>
+      </c>
+      <c r="D385" s="1"/>
+      <c r="E385" s="7" t="s">
+        <v>772</v>
+      </c>
+      <c r="F385" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="G385" s="26"/>
     </row>
     <row r="386" spans="1:7">
       <c r="A386" s="2" t="s">
-        <v>894</v>
+        <v>765</v>
       </c>
       <c r="B386" s="2" t="s">
-        <v>898</v>
+        <v>1014</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>899</v>
-      </c>
-      <c r="D386" s="7" t="s">
-        <v>900</v>
-      </c>
+        <v>1015</v>
+      </c>
+      <c r="D386" s="1"/>
       <c r="E386" s="7"/>
-      <c r="F386" s="4" t="s">
-        <v>20</v>
+      <c r="F386" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="G386" s="26"/>
     </row>
-    <row r="387" spans="1:7" ht="30">
+    <row r="387" spans="1:7">
       <c r="A387" s="2" t="s">
         <v>894</v>
       </c>
       <c r="B387" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="C387" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="D387" s="7" t="s">
+        <v>897</v>
+      </c>
+      <c r="E387" s="7"/>
+      <c r="F387" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="G387" s="26"/>
+    </row>
+    <row r="388" spans="1:7">
+      <c r="A388" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="B388" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="C388" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="D388" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="E388" s="7"/>
+      <c r="F388" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G388" s="26"/>
+    </row>
+    <row r="389" spans="1:7" ht="30">
+      <c r="A389" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="B389" s="2" t="s">
         <v>901</v>
       </c>
-      <c r="C387" s="2" t="s">
+      <c r="C389" s="2" t="s">
         <v>902</v>
       </c>
-      <c r="D387" s="1" t="s">
+      <c r="D389" s="1" t="s">
         <v>903</v>
       </c>
-      <c r="E387" s="7"/>
-      <c r="F387" s="4" t="s">
+      <c r="E389" s="7"/>
+      <c r="F389" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G387" s="26"/>
-    </row>
-    <row r="388" spans="1:7" ht="30">
-      <c r="A388" s="17" t="s">
+      <c r="G389" s="26"/>
+    </row>
+    <row r="390" spans="1:7" ht="30">
+      <c r="A390" s="17" t="s">
         <v>894</v>
       </c>
-      <c r="B388" s="17" t="s">
+      <c r="B390" s="17" t="s">
         <v>904</v>
       </c>
-      <c r="C388" s="17" t="s">
+      <c r="C390" s="17" t="s">
         <v>905</v>
       </c>
-      <c r="D388" s="27"/>
-      <c r="E388" s="27"/>
-      <c r="F388" s="18" t="s">
+      <c r="D390" s="27"/>
+      <c r="E390" s="27"/>
+      <c r="F390" s="18" t="s">
         <v>906</v>
       </c>
-      <c r="G388" s="28"/>
-    </row>
-    <row r="389" spans="1:7">
-      <c r="A389" t="s">
-        <v>894</v>
-      </c>
-      <c r="B389" t="s">
-        <v>907</v>
-      </c>
-      <c r="C389" t="s">
-        <v>908</v>
-      </c>
-      <c r="D389" s="7"/>
-      <c r="E389" s="7"/>
-      <c r="F389" t="s">
-        <v>29</v>
-      </c>
-      <c r="G389" s="26"/>
-    </row>
-    <row r="390" spans="1:7">
-      <c r="A390" t="s">
-        <v>894</v>
-      </c>
-      <c r="B390" t="s">
-        <v>909</v>
-      </c>
-      <c r="C390" t="s">
-        <v>910</v>
-      </c>
-      <c r="D390" s="7" t="s">
-        <v>911</v>
-      </c>
-      <c r="E390" s="7"/>
-      <c r="F390" t="s">
-        <v>29</v>
-      </c>
-      <c r="G390" s="26"/>
+      <c r="G390" s="28"/>
     </row>
     <row r="391" spans="1:7">
       <c r="A391" t="s">
         <v>894</v>
       </c>
       <c r="B391" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="C391" t="s">
-        <v>913</v>
-      </c>
-      <c r="D391" s="7" t="s">
-        <v>914</v>
-      </c>
+        <v>908</v>
+      </c>
+      <c r="D391" s="7"/>
       <c r="E391" s="7"/>
       <c r="F391" t="s">
+        <v>29</v>
+      </c>
+      <c r="G391" s="26"/>
+    </row>
+    <row r="392" spans="1:7">
+      <c r="A392" t="s">
+        <v>894</v>
+      </c>
+      <c r="B392" t="s">
+        <v>909</v>
+      </c>
+      <c r="C392" t="s">
+        <v>910</v>
+      </c>
+      <c r="D392" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="E392" s="7"/>
+      <c r="F392" t="s">
+        <v>29</v>
+      </c>
+      <c r="G392" s="26"/>
+    </row>
+    <row r="393" spans="1:7">
+      <c r="A393" t="s">
+        <v>894</v>
+      </c>
+      <c r="B393" t="s">
+        <v>912</v>
+      </c>
+      <c r="C393" t="s">
+        <v>913</v>
+      </c>
+      <c r="D393" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="E393" s="7"/>
+      <c r="F393" t="s">
         <v>20</v>
       </c>
-      <c r="G391" s="26"/>
-    </row>
-    <row r="392" spans="1:7">
-      <c r="D392" s="7"/>
-      <c r="E392" s="7"/>
-      <c r="G392" s="26"/>
+      <c r="G393" s="26"/>
+    </row>
+    <row r="394" spans="1:7">
+      <c r="D394" s="7"/>
+      <c r="E394" s="7"/>
+      <c r="G394" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>